<commit_message>
Add issue and return book transaction workflow
</commit_message>
<xml_diff>
--- a/library.xlsx
+++ b/library.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECTS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECTS\LibraryManagementSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BB896FF-B2A2-43FF-A8F2-B8EF59F54A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744348AF-9AC2-46B8-B1B3-E786A4164B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="690" windowWidth="15060" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11355" yWindow="615" windowWidth="15060" windowHeight="14790" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Members" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
   <si>
     <t>ইন্দ্রানী</t>
   </si>
@@ -135,6 +135,45 @@
   <si>
     <t>serial_no</t>
   </si>
+  <si>
+    <t>member_no</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>designation</t>
+  </si>
+  <si>
+    <t>department</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>M1001</t>
+  </si>
+  <si>
+    <t>Partha Sarkar</t>
+  </si>
+  <si>
+    <t>member</t>
+  </si>
+  <si>
+    <t>Chandanangore</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
 </sst>
 </file>
 
@@ -143,7 +182,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-5000445]0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -174,6 +213,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -240,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -324,6 +371,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -24378,9 +24426,56 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2">
+        <v>9674991301</v>
+      </c>
+      <c r="H2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
messages : route changed added
</commit_message>
<xml_diff>
--- a/library.xlsx
+++ b/library.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECTS\LibraryManagementSystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PYTHON_TUTORIAL\LibraryManagementSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744348AF-9AC2-46B8-B1B3-E786A4164B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4B2124-587B-4AEB-A5A1-898EB1F1B3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11355" yWindow="615" windowWidth="15060" windowHeight="14790" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="51">
   <si>
     <t>ইন্দ্রানী</t>
   </si>
@@ -173,6 +173,12 @@
   </si>
   <si>
     <t>Active</t>
+  </si>
+  <si>
+    <t>M1002</t>
+  </si>
+  <si>
+    <t>Pol Sarkar</t>
   </si>
 </sst>
 </file>
@@ -362,6 +368,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -371,7 +378,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14375,10 +14381,10 @@
       <c r="E3474" s="12"/>
     </row>
     <row r="3476" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D3476" s="32"/>
+      <c r="D3476" s="33"/>
     </row>
     <row r="3477" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D3477" s="32"/>
+      <c r="D3477" s="33"/>
     </row>
     <row r="3478" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3478" s="16"/>
@@ -16289,13 +16295,13 @@
       <c r="E4038" s="13"/>
     </row>
     <row r="4039" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4039" s="33"/>
-      <c r="C4039" s="34"/>
+      <c r="B4039" s="34"/>
+      <c r="C4039" s="35"/>
       <c r="E4039" s="13"/>
     </row>
     <row r="4040" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4040" s="33"/>
-      <c r="C4040" s="34"/>
+      <c r="B4040" s="34"/>
+      <c r="C4040" s="35"/>
       <c r="E4040" s="13"/>
     </row>
     <row r="4041" spans="2:5" x14ac:dyDescent="0.25">
@@ -16349,13 +16355,13 @@
       <c r="E4057" s="13"/>
     </row>
     <row r="4058" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4058" s="33"/>
-      <c r="C4058" s="34"/>
+      <c r="B4058" s="34"/>
+      <c r="C4058" s="35"/>
       <c r="E4058" s="13"/>
     </row>
     <row r="4059" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4059" s="33"/>
-      <c r="C4059" s="34"/>
+      <c r="B4059" s="34"/>
+      <c r="C4059" s="35"/>
       <c r="E4059" s="13"/>
     </row>
     <row r="4060" spans="2:5" x14ac:dyDescent="0.25">
@@ -22076,14 +22082,14 @@
       <c r="E5210" s="13"/>
     </row>
     <row r="5211" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5211" s="33"/>
+      <c r="B5211" s="34"/>
       <c r="C5211" s="4"/>
-      <c r="E5211" s="32"/>
+      <c r="E5211" s="33"/>
     </row>
     <row r="5212" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5212" s="33"/>
+      <c r="B5212" s="34"/>
       <c r="C5212" s="4"/>
-      <c r="E5212" s="32"/>
+      <c r="E5212" s="33"/>
     </row>
     <row r="5213" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5213" s="14"/>
@@ -24426,32 +24432,37 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="35" t="s">
+      <c r="G1" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="35" t="s">
+      <c r="H1" s="32" t="s">
         <v>43</v>
       </c>
     </row>
@@ -24475,6 +24486,26 @@
         <v>48</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3">
+        <v>8820496038</v>
+      </c>
+      <c r="H3" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve UI with logo, navbar, footer and dashboard updates
</commit_message>
<xml_diff>
--- a/library.xlsx
+++ b/library.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PYTHON_TUTORIAL\LibraryManagementSystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECTS\LibraryManagementSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4B2124-587B-4AEB-A5A1-898EB1F1B3CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFC7A17-65C5-4698-879E-013A9B62AA94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4995" yWindow="1875" windowWidth="17325" windowHeight="14790" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="54">
   <si>
     <t>ইন্দ্রানী</t>
   </si>
@@ -180,6 +180,15 @@
   <si>
     <t>Pol Sarkar</t>
   </si>
+  <si>
+    <t>Accts</t>
+  </si>
+  <si>
+    <t>par@gmail.com</t>
+  </si>
+  <si>
+    <t>par1@gmail.com</t>
+  </si>
 </sst>
 </file>
 
@@ -188,7 +197,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-5000445]0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,6 +236,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -290,10 +307,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -378,8 +396,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -24437,7 +24457,10 @@
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -24476,11 +24499,17 @@
       <c r="C2" t="s">
         <v>46</v>
       </c>
+      <c r="D2" t="s">
+        <v>51</v>
+      </c>
       <c r="E2" t="s">
         <v>47</v>
       </c>
       <c r="F2">
         <v>9674991301</v>
+      </c>
+      <c r="G2" s="36" t="s">
+        <v>52</v>
       </c>
       <c r="H2" t="s">
         <v>48</v>
@@ -24496,17 +24525,27 @@
       <c r="C3" t="s">
         <v>46</v>
       </c>
+      <c r="D3" t="s">
+        <v>51</v>
+      </c>
       <c r="E3" t="s">
         <v>47</v>
       </c>
       <c r="F3">
         <v>8820496038</v>
       </c>
+      <c r="G3" s="36" t="s">
+        <v>53</v>
+      </c>
       <c r="H3" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{6E4E2AA9-B6F6-49A0-9DEA-56B01142700C}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{DCF13848-0843-4846-9BEF-06D8F416A59A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>